<commit_message>
feat(arch): implement multi-crew autonomous trading framework and post-market safety wall
- Implement 5-crew architecture: PreMarketCrew, ScannerCrew, TradingCrew (with OrderFlowAgent), ExecutionCrew, and PostMarketCrew
- Implement Capital Safety Wall lock mechanism (50% daily reserve lock & institutional scaling)
- Add OrderFlowAgent for institutional bid/ask imbalances, iceberg absorption, and delta confluence
- Modularize live scanner with autonomous crew pipelines and post-market audit automation
- Add daily reporting orchestrator, risk configurations, and state persistence
- Update architecture documentation, SVG/PNG diagrams, PDFs, and documentation exports
- Add full test suite for multi-crew trading workflows
</commit_message>
<xml_diff>
--- a/trades/by_strategy/liquidity_sweep.xlsx
+++ b/trades/by_strategy/liquidity_sweep.xlsx
@@ -10,7 +10,7 @@
     <sheet xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" name="Liquidity Sweep" sheetId="1" state="visible" r:id="rId1"/>
   </sheets>
   <definedNames>
-    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Liquidity Sweep'!$A$1:$Z$8</definedName>
+    <definedName name="_xlnm._FilterDatabase" localSheetId="0" hidden="1">'Liquidity Sweep'!$A$1:$Z$6</definedName>
   </definedNames>
   <calcPr calcId="124519" fullCalcOnLoad="1"/>
 </workbook>
@@ -40,13 +40,13 @@
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="0015803D"/>
+      <color rgb="00B91C1C"/>
       <sz val="11"/>
     </font>
     <font>
       <name val="Calibri"/>
       <b val="1"/>
-      <color rgb="00B91C1C"/>
+      <color rgb="0015803D"/>
       <sz val="11"/>
     </font>
   </fonts>
@@ -96,7 +96,7 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="23">
+  <cellXfs count="19">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" pivotButton="0" quotePrefix="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="center" vertical="center" wrapText="1"/>
@@ -143,9 +143,6 @@
     <xf numFmtId="166" fontId="2" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
-    <xf numFmtId="166" fontId="0" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
     <xf numFmtId="164" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
@@ -153,15 +150,6 @@
       <alignment horizontal="right" vertical="center"/>
     </xf>
     <xf numFmtId="166" fontId="3" fillId="0" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="164" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="165" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
-      <alignment horizontal="right" vertical="center"/>
-    </xf>
-    <xf numFmtId="166" fontId="3" fillId="3" borderId="1" applyAlignment="1" pivotButton="0" quotePrefix="0" xfId="0">
       <alignment horizontal="right" vertical="center"/>
     </xf>
   </cellXfs>
@@ -529,13 +517,13 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:Z8"/>
+  <dimension ref="A1:Z6"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="13" customWidth="1" min="1" max="1"/>
     <col width="12" customWidth="1" min="2" max="2"/>
     <col width="18" customWidth="1" min="3" max="3"/>
-    <col width="38" customWidth="1" min="4" max="4"/>
+    <col width="57" customWidth="1" min="4" max="4"/>
     <col width="12" customWidth="1" min="5" max="5"/>
     <col width="20" customWidth="1" min="6" max="6"/>
     <col width="13" customWidth="1" min="7" max="7"/>
@@ -544,7 +532,7 @@
     <col width="12" customWidth="1" min="10" max="10"/>
     <col width="12" customWidth="1" min="11" max="11"/>
     <col width="12" customWidth="1" min="12" max="12"/>
-    <col width="28" customWidth="1" min="13" max="13"/>
+    <col width="49" customWidth="1" min="13" max="13"/>
     <col width="12" customWidth="1" min="14" max="14"/>
     <col width="13" customWidth="1" min="15" max="15"/>
     <col width="17" customWidth="1" min="16" max="16"/>
@@ -695,12 +683,12 @@
     <row r="2" ht="20" customHeight="1">
       <c r="A2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-08-06</t>
         </is>
       </c>
       <c r="B2" s="2" t="inlineStr">
         <is>
-          <t>10:25</t>
+          <t>13:10</t>
         </is>
       </c>
       <c r="C2" s="3" t="inlineStr">
@@ -710,7 +698,7 @@
       </c>
       <c r="D2" s="3" t="inlineStr">
         <is>
-          <t>Liquidity Sweep [Tier 1 (General]</t>
+          <t>Liquidity Sweep [Preferred Lot Size: 3 Lots (195 Qty)]</t>
         </is>
       </c>
       <c r="E2" s="2" t="inlineStr">
@@ -720,67 +708,67 @@
       </c>
       <c r="F2" s="2" t="inlineStr">
         <is>
-          <t>TRAILED (+1.88R)</t>
+          <t>STOPPED OUT (-1R)</t>
         </is>
       </c>
       <c r="G2" s="4" t="n">
-        <v>23444.1</v>
+        <v>24627.15</v>
       </c>
       <c r="H2" s="4" t="n">
-        <v>23475.6</v>
+        <v>24681.8</v>
       </c>
       <c r="I2" s="4" t="n">
-        <v>23320.15</v>
+        <v>24501.25</v>
       </c>
       <c r="J2" s="4" t="n">
-        <v>31.5</v>
+        <v>54.65</v>
       </c>
       <c r="K2" s="4" t="n">
-        <v>23388.65</v>
+        <v>24633.05</v>
       </c>
       <c r="L2" s="2" t="inlineStr">
         <is>
-          <t>11:00</t>
+          <t>13:45</t>
         </is>
       </c>
       <c r="M2" s="3" t="inlineStr">
         <is>
-          <t>Partial + Structure Trail</t>
+          <t>30-Min Stagnation Time-Stop (Theta Guard: 30m)</t>
         </is>
       </c>
       <c r="N2" s="4" t="n">
-        <v>55.45</v>
+        <v>-5.9</v>
       </c>
       <c r="O2" s="5" t="n">
-        <v>1.88</v>
+        <v>-0.11</v>
       </c>
       <c r="P2" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 23400 PE</t>
+          <t>NIFTY 24550 PE</t>
         </is>
       </c>
       <c r="Q2" s="2" t="inlineStr">
         <is>
-          <t>2026-09-29</t>
+          <t>2026-08-11</t>
         </is>
       </c>
       <c r="R2" s="4" t="n">
-        <v>126.76</v>
+        <v>104.6</v>
       </c>
       <c r="S2" s="4" t="n">
-        <v>153.08</v>
+        <v>101.87</v>
       </c>
       <c r="T2" s="6" t="n">
-        <v>24718</v>
+        <v>20397</v>
       </c>
       <c r="U2" s="6" t="n">
-        <v>29851</v>
+        <v>19865</v>
       </c>
       <c r="V2" s="7" t="n">
-        <v>5032</v>
+        <v>-617</v>
       </c>
       <c r="W2" s="8" t="n">
-        <v>20.4</v>
+        <v>-3</v>
       </c>
       <c r="X2" s="2" t="n">
         <v>3</v>
@@ -790,19 +778,19 @@
       </c>
       <c r="Z2" s="3" t="inlineStr">
         <is>
-          <t>09:20 sweep: 5m high 23,489.00 above PDH 23,466.65 | 09:30 rejection: 15m close 23,445.90 back below PDH 23,466.65 | 10:25 structure break: 5m close 23,444.10 below 5m swing low 23,449.55 (09:55) | 10:25 entry: 5m close 23,444.10 below VWAP, below PDH 23,466.65 and below the open 23,454.05 | 10:25 trendline breakdown: 5m close 23,444.10 below ascending trendline 23,469.34</t>
+          <t>11:30 sweep: 5m high 24,674.80 above PDH 24,669.20 | 11:45 rejection: 15m close 24,633.65 back below PDH 24,669.20 | 13:10 structure break: 5m close 24,627.15 below 5m swing low 24,627.20 (12:20) | 13:10 entry: 5m close 24,627.15 below VWAP, below PDH 24,669.20 and below the open 24,632.70</t>
         </is>
       </c>
     </row>
     <row r="3" ht="20" customHeight="1">
       <c r="A3" s="9" t="inlineStr">
         <is>
-          <t>2026-09-15</t>
+          <t>2026-08-18</t>
         </is>
       </c>
       <c r="B3" s="9" t="inlineStr">
         <is>
-          <t>10:30</t>
+          <t>09:30</t>
         </is>
       </c>
       <c r="C3" s="10" t="inlineStr">
@@ -812,77 +800,77 @@
       </c>
       <c r="D3" s="10" t="inlineStr">
         <is>
-          <t>Liquidity Sweep [Tier 1 (General]</t>
+          <t>Liquidity Sweep [Preferred Lot Size: 3 Lots (195 Qty)]</t>
         </is>
       </c>
       <c r="E3" s="9" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="F3" s="9" t="inlineStr">
         <is>
-          <t>TRAILED (+2.10R)</t>
+          <t>STOPPED OUT (-1R)</t>
         </is>
       </c>
       <c r="G3" s="11" t="n">
-        <v>23362.65</v>
+        <v>24245.1</v>
       </c>
       <c r="H3" s="11" t="n">
-        <v>23404.3</v>
+        <v>24209.6</v>
       </c>
       <c r="I3" s="11" t="n">
-        <v>23235.25</v>
+        <v>24356.9</v>
       </c>
       <c r="J3" s="11" t="n">
-        <v>41.65</v>
+        <v>35.5</v>
       </c>
       <c r="K3" s="11" t="n">
-        <v>23271.35</v>
+        <v>24222.8</v>
       </c>
       <c r="L3" s="9" t="inlineStr">
         <is>
-          <t>13:50</t>
+          <t>10:05</t>
         </is>
       </c>
       <c r="M3" s="10" t="inlineStr">
         <is>
-          <t>Partial + Structure Trail</t>
+          <t>30-Min Stagnation Time-Stop (Theta Guard: 30m)</t>
         </is>
       </c>
       <c r="N3" s="11" t="n">
-        <v>91.3</v>
+        <v>-22.3</v>
       </c>
       <c r="O3" s="12" t="n">
-        <v>2.1</v>
+        <v>-0.63</v>
       </c>
       <c r="P3" s="10" t="inlineStr">
         <is>
-          <t>NIFTY 23300 PE</t>
+          <t>NIFTY 24350 CE</t>
         </is>
       </c>
       <c r="Q3" s="9" t="inlineStr">
         <is>
-          <t>2026-09-22</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="R3" s="11" t="n">
-        <v>131.37</v>
+        <v>107.95</v>
       </c>
       <c r="S3" s="11" t="n">
-        <v>173.62</v>
+        <v>99.11</v>
       </c>
       <c r="T3" s="13" t="n">
-        <v>25617</v>
+        <v>21050</v>
       </c>
       <c r="U3" s="13" t="n">
-        <v>33856</v>
+        <v>19326</v>
       </c>
       <c r="V3" s="14" t="n">
-        <v>8132</v>
+        <v>-1808</v>
       </c>
       <c r="W3" s="15" t="n">
-        <v>31.7</v>
+        <v>-8.6</v>
       </c>
       <c r="X3" s="9" t="n">
         <v>3</v>
@@ -892,14 +880,14 @@
       </c>
       <c r="Z3" s="10" t="inlineStr">
         <is>
-          <t>09:20 sweep: 5m high 23,588.30 above PDH 23,447.90 | 10:00 rejection: 15m close 23,394.60 back below PDH 23,447.90 | 10:30 structure break: 5m close 23,362.65 below 5m swing low 23,369.80 (10:10) | 10:30 entry: 5m close 23,362.65 below VWAP, below PDH 23,447.90 and below the open 23,576.15</t>
+          <t>09:20 sweep: 5m low 24,214.60 below PDL 24,226.95 | 09:25 immediate reclaim: 5m close 24,244.35 snapped back above PDL | 09:30 entry: 5m close 24,245.10 above VWAP, above PDL 24,226.95 and above the open 24,223.05</t>
         </is>
       </c>
     </row>
     <row r="4" ht="20" customHeight="1">
       <c r="A4" s="2" t="inlineStr">
         <is>
-          <t>2026-08-26</t>
+          <t>2026-08-21</t>
         </is>
       </c>
       <c r="B4" s="2" t="inlineStr">
@@ -914,7 +902,7 @@
       </c>
       <c r="D4" s="3" t="inlineStr">
         <is>
-          <t>Liquidity Sweep [Tier 1 (General]</t>
+          <t>Liquidity Sweep [Preferred Lot Size: 3 Lots (195 Qty)]</t>
         </is>
       </c>
       <c r="E4" s="2" t="inlineStr">
@@ -924,77 +912,77 @@
       </c>
       <c r="F4" s="2" t="inlineStr">
         <is>
-          <t>TRAILED (+0.27R)</t>
+          <t>STOPPED OUT (-1R)</t>
         </is>
       </c>
       <c r="G4" s="4" t="n">
-        <v>24288.45</v>
+        <v>24239.3</v>
       </c>
       <c r="H4" s="4" t="n">
-        <v>24337.65</v>
+        <v>24287</v>
       </c>
       <c r="I4" s="4" t="n">
-        <v>24118.55</v>
+        <v>24096.2</v>
       </c>
       <c r="J4" s="4" t="n">
-        <v>49.2</v>
+        <v>47.7</v>
       </c>
       <c r="K4" s="4" t="n">
-        <v>24275.35</v>
+        <v>24243.1</v>
       </c>
       <c r="L4" s="2" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>12:35</t>
         </is>
       </c>
       <c r="M4" s="3" t="inlineStr">
         <is>
-          <t>Time (15:10)</t>
+          <t>30-Min Stagnation Time-Stop (Theta Guard: 30m)</t>
         </is>
       </c>
       <c r="N4" s="4" t="n">
-        <v>13.1</v>
+        <v>-3.8</v>
       </c>
       <c r="O4" s="5" t="n">
-        <v>0.27</v>
+        <v>-0.08</v>
       </c>
       <c r="P4" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 24250 PE</t>
+          <t>NIFTY 24150 PE</t>
         </is>
       </c>
       <c r="Q4" s="2" t="inlineStr">
         <is>
-          <t>2026-09-01</t>
+          <t>2026-08-25</t>
         </is>
       </c>
       <c r="R4" s="4" t="n">
-        <v>120.82</v>
+        <v>71.72</v>
       </c>
       <c r="S4" s="4" t="n">
-        <v>125.36</v>
+        <v>70.01000000000001</v>
       </c>
       <c r="T4" s="6" t="n">
-        <v>15707</v>
+        <v>13985</v>
       </c>
       <c r="U4" s="6" t="n">
-        <v>16297</v>
+        <v>13652</v>
       </c>
       <c r="V4" s="7" t="n">
-        <v>513</v>
+        <v>-406</v>
       </c>
       <c r="W4" s="8" t="n">
-        <v>3.3</v>
+        <v>-2.9</v>
       </c>
       <c r="X4" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y4" s="2" t="n">
-        <v>130</v>
+        <v>195</v>
       </c>
       <c r="Z4" s="3" t="inlineStr">
         <is>
-          <t>09:20 sweep: 5m high 24,355.35 above PDH 24,334.55 | 10:30 rejection: 15m close 24,304.60 back below PDH 24,334.55 | 11:55 structure break: 5m close 24,285.15 below 5m swing low 24,292.75 (11:30) | 11:55 entry: 5m close 24,285.15 below VWAP, below PDH 24,334.55 and below the open 24,343.05 | 12:00 entry: 5m close 24,288.45 below VWAP, below PDH 24,334.55 and below the open 24,343.05 | [Midday Waterfall Active (Tier parameters satisfied)]</t>
+          <t>09:20 sweep: 5m high 24,282.00 above PDH 24,263.95 | 09:30 rejection: 15m close 24,230.80 back below PDH 24,263.95 | 11:55 structure break: 5m close 24,245.25 below 5m swing low 24,248.15 (11:20) | 12:00 entry: 5m close 24,239.30 below VWAP, below PDH 24,263.95 and below the open 24,282.00 | 12:00 trendline breakdown: 5m close 24,239.30 below ascending trendline 24,259.93 | [Midday Waterfall Active (Tier parameters satisfied)]</t>
         </is>
       </c>
     </row>
@@ -1006,7 +994,7 @@
       </c>
       <c r="B5" s="9" t="inlineStr">
         <is>
-          <t>10:00</t>
+          <t>09:35</t>
         </is>
       </c>
       <c r="C5" s="10" t="inlineStr">
@@ -1016,7 +1004,7 @@
       </c>
       <c r="D5" s="10" t="inlineStr">
         <is>
-          <t>Liquidity Sweep [Tier 1 (General]</t>
+          <t>Liquidity Sweep [Preferred Lot Size: 3 Lots (195 Qty)]</t>
         </is>
       </c>
       <c r="E5" s="9" t="inlineStr">
@@ -1026,39 +1014,39 @@
       </c>
       <c r="F5" s="9" t="inlineStr">
         <is>
-          <t>TRAILED (+1.64R)</t>
+          <t>TRAILED (+0.14R)</t>
         </is>
       </c>
       <c r="G5" s="11" t="n">
-        <v>24268.2</v>
+        <v>24276.75</v>
       </c>
       <c r="H5" s="11" t="n">
         <v>24317.85</v>
       </c>
       <c r="I5" s="11" t="n">
-        <v>24119.25</v>
+        <v>24153.45</v>
       </c>
       <c r="J5" s="11" t="n">
-        <v>49.65</v>
+        <v>41.1</v>
       </c>
       <c r="K5" s="11" t="n">
-        <v>24186.8</v>
+        <v>24270.9</v>
       </c>
       <c r="L5" s="9" t="inlineStr">
         <is>
-          <t>11:45</t>
+          <t>10:10</t>
         </is>
       </c>
       <c r="M5" s="10" t="inlineStr">
         <is>
-          <t>Structure Trail</t>
+          <t>30-Min Stagnation Time-Stop (Theta Guard: 30m)</t>
         </is>
       </c>
       <c r="N5" s="11" t="n">
-        <v>81.40000000000001</v>
-      </c>
-      <c r="O5" s="12" t="n">
-        <v>1.64</v>
+        <v>5.85</v>
+      </c>
+      <c r="O5" s="16" t="n">
+        <v>0.14</v>
       </c>
       <c r="P5" s="10" t="inlineStr">
         <is>
@@ -1071,44 +1059,44 @@
         </is>
       </c>
       <c r="R5" s="11" t="n">
-        <v>34.54</v>
+        <v>32.18</v>
       </c>
       <c r="S5" s="11" t="n">
-        <v>67.67</v>
+        <v>33.49</v>
       </c>
       <c r="T5" s="13" t="n">
-        <v>4490</v>
+        <v>6275</v>
       </c>
       <c r="U5" s="13" t="n">
-        <v>8797</v>
-      </c>
-      <c r="V5" s="14" t="n">
-        <v>4245</v>
-      </c>
-      <c r="W5" s="15" t="n">
-        <v>94.5</v>
+        <v>6531</v>
+      </c>
+      <c r="V5" s="17" t="n">
+        <v>196</v>
+      </c>
+      <c r="W5" s="18" t="n">
+        <v>3.1</v>
       </c>
       <c r="X5" s="9" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y5" s="9" t="n">
-        <v>130</v>
+        <v>195</v>
       </c>
       <c r="Z5" s="10" t="inlineStr">
         <is>
-          <t>09:20 sweep: 5m high 24,312.85 above PDH 24,282.00 | 09:45 rejection: 15m close 24,281.75 back below PDH 24,282.00 | 10:00 structure break: 5m close 24,268.20 below 5m swing low 24,272.55 (09:30) | 10:00 entry: 5m close 24,268.20 below VWAP, below PDH 24,282.00 and below the open 24,285.05</t>
+          <t>09:20 sweep: 5m high 24,312.85 above PDH 24,282.00 | 09:35 immediate reclaim: 5m close 24,276.75 snapped back below PDH | 09:35 entry: 5m close 24,276.75 below VWAP, below PDH 24,282.00 and below the open 24,285.05</t>
         </is>
       </c>
     </row>
     <row r="6" ht="20" customHeight="1">
       <c r="A6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-21</t>
+          <t>2026-09-10</t>
         </is>
       </c>
       <c r="B6" s="2" t="inlineStr">
         <is>
-          <t>12:00</t>
+          <t>10:45</t>
         </is>
       </c>
       <c r="C6" s="3" t="inlineStr">
@@ -1118,296 +1106,92 @@
       </c>
       <c r="D6" s="3" t="inlineStr">
         <is>
-          <t>Liquidity Sweep [Tier 1 (General]</t>
+          <t>Liquidity Sweep [Preferred Lot Size: 3 Lots (195 Qty)]</t>
         </is>
       </c>
       <c r="E6" s="2" t="inlineStr">
         <is>
-          <t>SHORT</t>
+          <t>LONG</t>
         </is>
       </c>
       <c r="F6" s="2" t="inlineStr">
         <is>
-          <t>TRAILED (+0.16R)</t>
+          <t>STOPPED OUT (-1R)</t>
         </is>
       </c>
       <c r="G6" s="4" t="n">
-        <v>24239.3</v>
+        <v>23448</v>
       </c>
       <c r="H6" s="4" t="n">
-        <v>24272.65</v>
+        <v>23399.4</v>
       </c>
       <c r="I6" s="4" t="n">
-        <v>24139.25</v>
+        <v>23568.35</v>
       </c>
       <c r="J6" s="4" t="n">
-        <v>33.35</v>
+        <v>48.6</v>
       </c>
       <c r="K6" s="4" t="n">
-        <v>24234.05</v>
+        <v>23436.75</v>
       </c>
       <c r="L6" s="2" t="inlineStr">
         <is>
-          <t>15:10</t>
+          <t>11:20</t>
         </is>
       </c>
       <c r="M6" s="3" t="inlineStr">
         <is>
-          <t>Time (15:10)</t>
+          <t>30-Min Stagnation Time-Stop (Theta Guard: 30m)</t>
         </is>
       </c>
       <c r="N6" s="4" t="n">
-        <v>5.25</v>
+        <v>-11.25</v>
       </c>
       <c r="O6" s="5" t="n">
-        <v>0.16</v>
+        <v>-0.23</v>
       </c>
       <c r="P6" s="3" t="inlineStr">
         <is>
-          <t>NIFTY 24200 PE</t>
+          <t>NIFTY 23550 CE</t>
         </is>
       </c>
       <c r="Q6" s="2" t="inlineStr">
         <is>
-          <t>2026-08-25</t>
+          <t>2026-09-15</t>
         </is>
       </c>
       <c r="R6" s="4" t="n">
-        <v>92.26000000000001</v>
+        <v>88.51000000000001</v>
       </c>
       <c r="S6" s="4" t="n">
-        <v>92.83</v>
+        <v>83.98</v>
       </c>
       <c r="T6" s="6" t="n">
-        <v>11994</v>
+        <v>17259</v>
       </c>
       <c r="U6" s="6" t="n">
-        <v>12068</v>
+        <v>16376</v>
       </c>
       <c r="V6" s="7" t="n">
-        <v>4</v>
-      </c>
-      <c r="W6" s="16" t="n">
-        <v>0</v>
+        <v>-961</v>
+      </c>
+      <c r="W6" s="8" t="n">
+        <v>-5.6</v>
       </c>
       <c r="X6" s="2" t="n">
-        <v>2</v>
+        <v>3</v>
       </c>
       <c r="Y6" s="2" t="n">
-        <v>130</v>
+        <v>195</v>
       </c>
       <c r="Z6" s="3" t="inlineStr">
         <is>
-          <t>09:20 sweep: 5m high 24,282.00 above PDH 24,263.95 | 09:30 rejection: 15m close 24,230.80 back below PDH 24,263.95 | 11:55 structure break: 5m close 24,245.25 below 5m swing low 24,248.15 (11:20) | 12:00 entry: 5m close 24,239.30 below VWAP, below PDH 24,263.95 and below the open 24,282.00 | 12:00 trendline breakdown: 5m close 24,239.30 below ascending trendline 24,259.93 | [Midday Waterfall Active (Tier parameters satisfied)]</t>
-        </is>
-      </c>
-    </row>
-    <row r="7" ht="20" customHeight="1">
-      <c r="A7" s="9" t="inlineStr">
-        <is>
-          <t>2026-08-06</t>
-        </is>
-      </c>
-      <c r="B7" s="9" t="inlineStr">
-        <is>
-          <t>13:10</t>
-        </is>
-      </c>
-      <c r="C7" s="10" t="inlineStr">
-        <is>
-          <t>Liquidity Sweep</t>
-        </is>
-      </c>
-      <c r="D7" s="10" t="inlineStr">
-        <is>
-          <t>Liquidity Sweep [Tier 1 (General]</t>
-        </is>
-      </c>
-      <c r="E7" s="9" t="inlineStr">
-        <is>
-          <t>SHORT</t>
-        </is>
-      </c>
-      <c r="F7" s="9" t="inlineStr">
-        <is>
-          <t>FLAT</t>
-        </is>
-      </c>
-      <c r="G7" s="11" t="n">
-        <v>24627.15</v>
-      </c>
-      <c r="H7" s="11" t="n">
-        <v>24681.8</v>
-      </c>
-      <c r="I7" s="11" t="n">
-        <v>24501.25</v>
-      </c>
-      <c r="J7" s="11" t="n">
-        <v>54.65</v>
-      </c>
-      <c r="K7" s="11" t="n">
-        <v>24628.2</v>
-      </c>
-      <c r="L7" s="9" t="inlineStr">
-        <is>
-          <t>15:10</t>
-        </is>
-      </c>
-      <c r="M7" s="10" t="inlineStr">
-        <is>
-          <t>Time (15:10)</t>
-        </is>
-      </c>
-      <c r="N7" s="11" t="n">
-        <v>-1.05</v>
-      </c>
-      <c r="O7" s="17" t="n">
-        <v>-0.02</v>
-      </c>
-      <c r="P7" s="10" t="inlineStr">
-        <is>
-          <t>NIFTY 24600 PE</t>
-        </is>
-      </c>
-      <c r="Q7" s="9" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="R7" s="11" t="n">
-        <v>126.79</v>
-      </c>
-      <c r="S7" s="11" t="n">
-        <v>125.15</v>
-      </c>
-      <c r="T7" s="13" t="n">
-        <v>16483</v>
-      </c>
-      <c r="U7" s="13" t="n">
-        <v>16270</v>
-      </c>
-      <c r="V7" s="18" t="n">
-        <v>-291</v>
-      </c>
-      <c r="W7" s="19" t="n">
-        <v>-1.8</v>
-      </c>
-      <c r="X7" s="9" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y7" s="9" t="n">
-        <v>130</v>
-      </c>
-      <c r="Z7" s="10" t="inlineStr">
-        <is>
-          <t>11:30 sweep: 5m high 24,674.80 above PDH 24,669.20 | 11:45 rejection: 15m close 24,633.65 back below PDH 24,669.20 | 13:10 structure break: 5m close 24,627.15 below 5m swing low 24,627.20 (12:20) | 13:10 entry: 5m close 24,627.15 below VWAP, below PDH 24,669.20 and below the open 24,632.70</t>
-        </is>
-      </c>
-    </row>
-    <row r="8" ht="20" customHeight="1">
-      <c r="A8" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-05</t>
-        </is>
-      </c>
-      <c r="B8" s="2" t="inlineStr">
-        <is>
-          <t>09:55</t>
-        </is>
-      </c>
-      <c r="C8" s="3" t="inlineStr">
-        <is>
-          <t>Liquidity Sweep</t>
-        </is>
-      </c>
-      <c r="D8" s="3" t="inlineStr">
-        <is>
-          <t>Liquidity Sweep [Tier 3 (Expensive]</t>
-        </is>
-      </c>
-      <c r="E8" s="2" t="inlineStr">
-        <is>
-          <t>SHORT</t>
-        </is>
-      </c>
-      <c r="F8" s="2" t="inlineStr">
-        <is>
-          <t>STOPPED OUT (-1R)</t>
-        </is>
-      </c>
-      <c r="G8" s="4" t="n">
-        <v>24591.2</v>
-      </c>
-      <c r="H8" s="4" t="n">
-        <v>24640.95</v>
-      </c>
-      <c r="I8" s="4" t="n">
-        <v>24431.2</v>
-      </c>
-      <c r="J8" s="4" t="n">
-        <v>49.75</v>
-      </c>
-      <c r="K8" s="4" t="n">
-        <v>24640.95</v>
-      </c>
-      <c r="L8" s="2" t="inlineStr">
-        <is>
-          <t>11:00</t>
-        </is>
-      </c>
-      <c r="M8" s="3" t="inlineStr">
-        <is>
-          <t>Stop</t>
-        </is>
-      </c>
-      <c r="N8" s="4" t="n">
-        <v>-49.75</v>
-      </c>
-      <c r="O8" s="20" t="n">
-        <v>-1</v>
-      </c>
-      <c r="P8" s="3" t="inlineStr">
-        <is>
-          <t>NIFTY 24550 PE</t>
-        </is>
-      </c>
-      <c r="Q8" s="2" t="inlineStr">
-        <is>
-          <t>2026-08-11</t>
-        </is>
-      </c>
-      <c r="R8" s="4" t="n">
-        <v>136.4</v>
-      </c>
-      <c r="S8" s="4" t="n">
-        <v>114.46</v>
-      </c>
-      <c r="T8" s="6" t="n">
-        <v>17732</v>
-      </c>
-      <c r="U8" s="6" t="n">
-        <v>14880</v>
-      </c>
-      <c r="V8" s="21" t="n">
-        <v>-2928</v>
-      </c>
-      <c r="W8" s="22" t="n">
-        <v>-16.5</v>
-      </c>
-      <c r="X8" s="2" t="n">
-        <v>2</v>
-      </c>
-      <c r="Y8" s="2" t="n">
-        <v>130</v>
-      </c>
-      <c r="Z8" s="3" t="inlineStr">
-        <is>
-          <t>09:20 sweep: 5m high 24,669.20 above PDH 24,666.65 | 09:30 rejection: 15m close 24,621.45 back below PDH 24,666.65 | 09:55 structure break: 5m close 24,591.20 below 5m swing low 24,604.95 (09:35) | 09:55 entry: 5m close 24,591.20 below VWAP, below PDH 24,666.65 and below the open 24,669.20</t>
+          <t>09:25 sweep: 5m low 23,414.40 below PDL 23,431.50 | 10:45 immediate reclaim: 5m close 23,448.00 snapped back above PDL | 10:45 entry: 5m close 23,448.00 above VWAP, above PDL 23,431.50 and above the open 23,446.60 | 10:45 trendline breakout: 5m close 23,448.00 above descending trendline 23,420.10</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <autoFilter ref="A1:Z8"/>
+  <autoFilter ref="A1:Z6"/>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
 </file>
</xml_diff>